<commit_message>
Mass changes to schematic pages - removal of components and traces from PCM - not yet attempted to update
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA_P2\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7303BEFE-5C1C-4419-B28B-4DC8D3D7B216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D291B4E1-02BB-4752-BAEE-0D3CDA3FD398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="245">
   <si>
     <t>G13</t>
   </si>
@@ -359,9 +359,6 @@
     <t>3V3</t>
   </si>
   <si>
-    <t>SIGNAL</t>
-  </si>
-  <si>
     <t>J6.5</t>
   </si>
   <si>
@@ -476,18 +473,9 @@
     <t>UART_TX</t>
   </si>
   <si>
-    <t>Debug Port UART RX</t>
-  </si>
-  <si>
-    <t>Debug Port UART TX</t>
-  </si>
-  <si>
     <t>USD_CSn[0]</t>
   </si>
   <si>
-    <t>uSD Chip Select</t>
-  </si>
-  <si>
     <t>USD_MOSI</t>
   </si>
   <si>
@@ -524,18 +512,6 @@
     <t>Power</t>
   </si>
   <si>
-    <t>ADC_CS_n</t>
-  </si>
-  <si>
-    <t>ADC CS active low</t>
-  </si>
-  <si>
-    <t>ADC_SCLK</t>
-  </si>
-  <si>
-    <t>ADC SCLK (rising edge active)</t>
-  </si>
-  <si>
     <t>ADC_MISO_A</t>
   </si>
   <si>
@@ -578,15 +554,6 @@
     <t>Audio PWM = A_SIG on schematic</t>
   </si>
   <si>
-    <t>Not used (Data 1 on schematic)</t>
-  </si>
-  <si>
-    <t>Not used (Data 2 on schematic)</t>
-  </si>
-  <si>
-    <t>AUDIO_EN</t>
-  </si>
-  <si>
     <t>ARTY A7 J4 CONNECTOR</t>
   </si>
   <si>
@@ -596,15 +563,6 @@
     <t>Signal Select 1=BNC, 0=Oscillator (gpio2_io_o_0[7])</t>
   </si>
   <si>
-    <t>IOX_SCLK</t>
-  </si>
-  <si>
-    <t>IOX_MOSI</t>
-  </si>
-  <si>
-    <t>IO Expander common SPI SCLK</t>
-  </si>
-  <si>
     <t>IOX_RESET</t>
   </si>
   <si>
@@ -635,9 +593,6 @@
     <t>IO Expander 2 Interrupt</t>
   </si>
   <si>
-    <t>IO Expander common SPI MOSI</t>
-  </si>
-  <si>
     <t>J4.13</t>
   </si>
   <si>
@@ -677,9 +632,6 @@
     <t>ADC_IP_IRQ</t>
   </si>
   <si>
-    <t>ADC PRIMARY IRQ</t>
-  </si>
-  <si>
     <t>CK_IO6</t>
   </si>
   <si>
@@ -737,35 +689,95 @@
     <t>UI_CSn</t>
   </si>
   <si>
-    <t>gpio2_io_o_0[9]</t>
-  </si>
-  <si>
-    <t>TEST_IO_0 (TP4 on PCB)</t>
-  </si>
-  <si>
-    <t>gpio2_io_o_0[0]</t>
-  </si>
-  <si>
-    <t>gpio2_io_o_0[1]</t>
-  </si>
-  <si>
-    <t>Timer 1 Test Signal ] = TIMER_1_OUTPUT) - TP6 ON PCB</t>
-  </si>
-  <si>
-    <t>Timer 2 Test Signal  =  TIMER_2_OUTPUT) - TP7 ON PCB</t>
-  </si>
-  <si>
     <t>ADC_IRQ_N_DONE</t>
   </si>
   <si>
     <t>gpio2_io_o_0[5]: N number of conversions done - indirect IRQ for ADC IP 7476Ax2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOFTCORE SA PHASE 2 </t>
+  </si>
+  <si>
+    <t>DIGILENT ARTY A7 TO IMR-107-SCH PIN MAP</t>
+  </si>
+  <si>
+    <t>IO Expander &amp; GP common SPI SCLK</t>
+  </si>
+  <si>
+    <t>IO Expander &amp; GP common SPI MOSI</t>
+  </si>
+  <si>
+    <t>IOX_GP_SCLK</t>
+  </si>
+  <si>
+    <t>IOX_GP_MOSI</t>
+  </si>
+  <si>
+    <t>Programmable Waveform Generator Chip Select / FSYNC</t>
+  </si>
+  <si>
+    <t>FSYNC</t>
+  </si>
+  <si>
+    <t>uSD Chip Insert Detect</t>
+  </si>
+  <si>
+    <t>A_EN</t>
+  </si>
+  <si>
+    <t>Debug Port UART RX - DBG_RX on schematic</t>
+  </si>
+  <si>
+    <t>Debug Port UART TX - DBG_TX on schematic</t>
+  </si>
+  <si>
+    <t>MCLK</t>
+  </si>
+  <si>
+    <t>ADC_CS_A</t>
+  </si>
+  <si>
+    <t>ADC_SCLK_A</t>
+  </si>
+  <si>
+    <t>ADC_CS_B</t>
+  </si>
+  <si>
+    <t>ADC_SCLK_B</t>
+  </si>
+  <si>
+    <t>ADC A CS active low</t>
+  </si>
+  <si>
+    <t>ADC A SCLK</t>
+  </si>
+  <si>
+    <t>ADC B CH active low</t>
+  </si>
+  <si>
+    <t>Programmable Waveform Generator MCLK 25MHz</t>
+  </si>
+  <si>
+    <t>ADC B SCLK</t>
+  </si>
+  <si>
+    <t>Wired on schematic but not used (DAT1 on schematic)</t>
+  </si>
+  <si>
+    <t>Wired on schematic but not used (DAT2 on schematic)</t>
+  </si>
+  <si>
+    <t>SIGNAL SCH</t>
+  </si>
+  <si>
+    <t>SIGNAL FPGA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -783,6 +795,22 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FF0070C0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -838,17 +866,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1183,17 +1213,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AF3F25-4127-44F5-ACE1-35E82582D3CE}">
-  <dimension ref="A4:I65"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" customWidth="1"/>
+    <col min="4" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="A1" s="7" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>64</v>
@@ -1202,28 +1242,32 @@
         <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>107</v>
+        <v>243</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="H4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="H5" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>244</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="I5" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1234,16 +1278,19 @@
         <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E6" t="s">
-        <v>163</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="F6" t="s">
+        <v>236</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1254,16 +1301,19 @@
         <v>92</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E7" t="s">
-        <v>167</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F7" t="s">
+        <v>159</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1274,19 +1324,22 @@
         <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E8" t="s">
-        <v>169</v>
-      </c>
-      <c r="H8" t="s">
-        <v>172</v>
+        <v>233</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F8" t="s">
+        <v>237</v>
       </c>
       <c r="I8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+      <c r="J8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1297,35 +1350,40 @@
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F9" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>100</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1336,13 +1394,16 @@
         <v>95</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="E12" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="F12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1353,13 +1414,16 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1370,13 +1434,16 @@
         <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="E14" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F14" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1387,13 +1454,16 @@
         <v>98</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E15" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -1403,8 +1473,9 @@
       <c r="D16" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>102</v>
       </c>
@@ -1414,17 +1485,19 @@
       <c r="D17" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1435,13 +1508,16 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F19" t="s">
         <v>148</v>
       </c>
-      <c r="E19" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1452,13 +1528,16 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="E20" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F20" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1469,13 +1548,16 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E21" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F21" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1486,35 +1568,40 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E22" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="9"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1524,11 +1611,11 @@
       <c r="C25" t="s">
         <v>87</v>
       </c>
-      <c r="E25" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1538,11 +1625,11 @@
       <c r="C26" t="s">
         <v>88</v>
       </c>
-      <c r="E26" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1553,13 +1640,14 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="E27" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1570,44 +1658,48 @@
         <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E28" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C30" t="s">
         <v>113</v>
-      </c>
-      <c r="C30" t="s">
-        <v>114</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1618,13 +1710,16 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E32" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F32" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -1635,13 +1730,16 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E33" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F33" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1652,13 +1750,14 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E34" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -1669,35 +1768,38 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E35" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="9"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1707,11 +1809,15 @@
       <c r="C38" t="s">
         <v>79</v>
       </c>
-      <c r="E38" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D38" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -1722,13 +1828,14 @@
         <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="E39" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+      <c r="E39" s="3"/>
+      <c r="F39" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -1739,13 +1846,14 @@
         <v>81</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="E40" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1756,44 +1864,48 @@
         <v>82</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E41" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C42" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="9"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C43" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="9"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -1804,13 +1916,14 @@
         <v>66</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E45" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -1821,13 +1934,14 @@
         <v>67</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E46" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -1838,13 +1952,14 @@
         <v>68</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E47" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -1855,15 +1970,16 @@
         <v>69</v>
       </c>
       <c r="D48" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s">
         <v>140</v>
       </c>
-      <c r="E48" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C49" t="s">
         <v>70</v>
@@ -1871,19 +1987,21 @@
       <c r="D49" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="9"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C50" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="9"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -1894,13 +2012,14 @@
         <v>71</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E51" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+      <c r="E51" s="3"/>
+      <c r="F51" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -1911,13 +2030,14 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E52" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -1928,13 +2048,14 @@
         <v>73</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+      <c r="E53" s="2"/>
+      <c r="F53" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1945,186 +2066,198 @@
         <v>74</v>
       </c>
       <c r="D54" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" t="s">
         <v>142</v>
       </c>
-      <c r="E54" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C55" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="9"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="9"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>66</v>
       </c>
       <c r="B58" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="C58" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="E58" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="C59" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E59" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C60" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="E60" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="5"/>
+      <c r="F60" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C61" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="E61" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C62" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="E62" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="C63" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="E63" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+      <c r="E63" s="2"/>
+      <c r="F63" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>185</v>
+      </c>
+      <c r="B64" t="s">
         <v>200</v>
       </c>
-      <c r="B64" t="s">
-        <v>216</v>
-      </c>
       <c r="C64" t="s">
+        <v>198</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E64" s="2"/>
+      <c r="F64" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>186</v>
+      </c>
+      <c r="B65" t="s">
+        <v>201</v>
+      </c>
+      <c r="C65" t="s">
+        <v>199</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D64" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E64" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>201</v>
-      </c>
-      <c r="B65" t="s">
-        <v>217</v>
-      </c>
-      <c r="C65" t="s">
-        <v>215</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="E65" t="s">
-        <v>219</v>
+      <c r="E65" s="2"/>
+      <c r="F65" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Routing done and clean up done - clean DRC - just letting it sit will review over the next 3 days before I release
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA_P2\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D291B4E1-02BB-4752-BAEE-0D3CDA3FD398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1AB282-4FCA-4169-8947-C95D0F8E625E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="261">
   <si>
     <t>G13</t>
   </si>
@@ -524,9 +524,6 @@
     <t>ADC B MISO</t>
   </si>
   <si>
-    <t>SIG_SEL</t>
-  </si>
-  <si>
     <t>Legend:</t>
   </si>
   <si>
@@ -551,9 +548,6 @@
     <t>AUDIO_PWM</t>
   </si>
   <si>
-    <t>Audio PWM = A_SIG on schematic</t>
-  </si>
-  <si>
     <t>ARTY A7 J4 CONNECTOR</t>
   </si>
   <si>
@@ -563,9 +557,6 @@
     <t>Signal Select 1=BNC, 0=Oscillator (gpio2_io_o_0[7])</t>
   </si>
   <si>
-    <t>IOX_RESET</t>
-  </si>
-  <si>
     <t>IO Expander common Reset (active low)</t>
   </si>
   <si>
@@ -581,9 +572,6 @@
     <t>IO Expander 2 chip select (active low)</t>
   </si>
   <si>
-    <t>IOX_MISO</t>
-  </si>
-  <si>
     <t>IO Expander common SPI MISO</t>
   </si>
   <si>
@@ -771,6 +759,66 @@
   </si>
   <si>
     <t>SIGNAL FPGA</t>
+  </si>
+  <si>
+    <t>S_SEL</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>MOSI</t>
+  </si>
+  <si>
+    <t>MISO</t>
+  </si>
+  <si>
+    <t>SCLK</t>
+  </si>
+  <si>
+    <t>DAT1</t>
+  </si>
+  <si>
+    <t>DAT2</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>1. If no label on schematic use FPGA signal name for both</t>
+  </si>
+  <si>
+    <t>DBG_RX</t>
+  </si>
+  <si>
+    <t>DBG_TX</t>
+  </si>
+  <si>
+    <t>A_PWM</t>
+  </si>
+  <si>
+    <t>Audio PWM</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[6]</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[8]</t>
+  </si>
+  <si>
+    <t>IOX_GP_MISO</t>
+  </si>
+  <si>
+    <t>X_SCLK</t>
+  </si>
+  <si>
+    <t>X_MOSI</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[7]</t>
   </si>
 </sst>
 </file>
@@ -873,12 +921,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1222,13 +1270,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A1" s="7" t="s">
-        <v>219</v>
+      <c r="A1" s="6" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>220</v>
+      <c r="A2" s="7" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -1242,27 +1290,27 @@
         <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>132</v>
       </c>
       <c r="I4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="A5" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
       <c r="I5" s="3" t="s">
         <v>155</v>
       </c>
@@ -1278,13 +1326,13 @@
         <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F6" t="s">
         <v>232</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F6" t="s">
-        <v>236</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>156</v>
@@ -1324,19 +1372,19 @@
         <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8" t="s">
         <v>233</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F8" t="s">
-        <v>237</v>
-      </c>
       <c r="I8" t="s">
+        <v>163</v>
+      </c>
+      <c r="J8" t="s">
         <v>164</v>
-      </c>
-      <c r="J8" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1350,13 +1398,13 @@
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F9" t="s">
         <v>234</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F9" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1369,7 +1417,9 @@
       <c r="D10" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E10" s="9"/>
+      <c r="I10" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1381,7 +1431,9 @@
       <c r="D11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="9"/>
+      <c r="I11" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1394,13 +1446,13 @@
         <v>95</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="F12" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1414,13 +1466,13 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>162</v>
+        <v>241</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>162</v>
+        <v>260</v>
       </c>
       <c r="F13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1434,13 +1486,13 @@
         <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="F14" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1473,7 +1525,6 @@
       <c r="D16" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E16" s="9"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1485,17 +1536,16 @@
       <c r="D17" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E17" s="9"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="A18" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1508,7 +1558,7 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>145</v>
+        <v>242</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>145</v>
@@ -1528,7 +1578,7 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>146</v>
+        <v>243</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>146</v>
@@ -1548,7 +1598,7 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>149</v>
@@ -1568,7 +1618,7 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>151</v>
+        <v>245</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>151</v>
@@ -1587,7 +1637,6 @@
       <c r="D23" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="9"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1599,7 +1648,6 @@
       <c r="D24" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E24" s="9"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1611,8 +1659,11 @@
       <c r="C25" t="s">
         <v>87</v>
       </c>
+      <c r="D25" t="s">
+        <v>246</v>
+      </c>
       <c r="F25" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1625,8 +1676,11 @@
       <c r="C26" t="s">
         <v>88</v>
       </c>
+      <c r="D26" t="s">
+        <v>247</v>
+      </c>
       <c r="F26" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1640,11 +1694,13 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E27" s="3"/>
       <c r="F27" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1658,11 +1714,13 @@
         <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="E28" s="2"/>
+        <v>222</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>222</v>
+      </c>
       <c r="F28" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1675,7 +1733,6 @@
       <c r="D29" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E29" s="9"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1687,17 +1744,16 @@
       <c r="D30" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="9"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="A31" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -1710,13 +1766,13 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="F32" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1730,13 +1786,13 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="F33" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1750,11 +1806,13 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E34" s="3"/>
+        <v>257</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="F34" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1768,11 +1826,13 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E35" s="2"/>
+        <v>256</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="F35" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1785,7 +1845,6 @@
       <c r="D36" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E36" s="9"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -1797,7 +1856,6 @@
       <c r="D37" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E37" s="9"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
@@ -1810,11 +1868,13 @@
         <v>79</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="E38" s="2"/>
+        <v>224</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="F38" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1828,11 +1888,11 @@
         <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1846,11 +1906,11 @@
         <v>81</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1864,11 +1924,11 @@
         <v>82</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1881,7 +1941,6 @@
       <c r="D42" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E42" s="9"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
@@ -1893,17 +1952,16 @@
       <c r="D43" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="9"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
+      <c r="A44" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -1918,7 +1976,9 @@
       <c r="D45" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E45" s="2"/>
+      <c r="E45" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="F45" t="s">
         <v>136</v>
       </c>
@@ -1936,7 +1996,9 @@
       <c r="D46" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E46" s="2"/>
+      <c r="E46" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="F46" t="s">
         <v>137</v>
       </c>
@@ -1954,7 +2016,9 @@
       <c r="D47" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E47" s="2"/>
+      <c r="E47" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="F47" t="s">
         <v>138</v>
       </c>
@@ -1972,7 +2036,9 @@
       <c r="D48" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E48" s="2"/>
+      <c r="E48" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="F48" t="s">
         <v>140</v>
       </c>
@@ -1987,7 +2053,6 @@
       <c r="D49" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E49" s="9"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -1999,7 +2064,6 @@
       <c r="D50" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E50" s="9"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
@@ -2011,12 +2075,14 @@
       <c r="C51" t="s">
         <v>71</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="E51" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E51" s="3"/>
       <c r="F51" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2030,11 +2096,13 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E52" s="2"/>
       <c r="F52" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2048,11 +2116,13 @@
         <v>73</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E53" s="2"/>
+        <v>253</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>169</v>
+      </c>
       <c r="F53" t="s">
-        <v>171</v>
+        <v>254</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2068,7 +2138,9 @@
       <c r="D54" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E54" s="2"/>
+      <c r="E54" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="F54" t="s">
         <v>142</v>
       </c>
@@ -2083,7 +2155,6 @@
       <c r="D55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E55" s="9"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
@@ -2095,34 +2166,33 @@
       <c r="D56" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E56" s="9"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="6"/>
+      <c r="A57" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>66</v>
       </c>
       <c r="B58" t="s">
+        <v>202</v>
+      </c>
+      <c r="C58" t="s">
+        <v>203</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="C58" t="s">
-        <v>207</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2130,17 +2200,17 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C59" t="s">
+        <v>201</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2148,17 +2218,17 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C60" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2166,17 +2236,17 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C61" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E61" s="5"/>
       <c r="F61" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2184,17 +2254,17 @@
         <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C62" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2202,53 +2272,53 @@
         <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C63" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B64" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C64" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C65" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Minor changes to text in SCH and PCB. DRC Good - Output Generation Complete
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA_P2\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1AB282-4FCA-4169-8947-C95D0F8E625E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D09CBD-13FA-4135-8F34-5E553F38B417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="281">
   <si>
     <t>G13</t>
   </si>
@@ -749,12 +749,6 @@
     <t>ADC B SCLK</t>
   </si>
   <si>
-    <t>Wired on schematic but not used (DAT1 on schematic)</t>
-  </si>
-  <si>
-    <t>Wired on schematic but not used (DAT2 on schematic)</t>
-  </si>
-  <si>
     <t>SIGNAL SCH</t>
   </si>
   <si>
@@ -819,6 +813,72 @@
   </si>
   <si>
     <t>gpio2_io_o_0[7]</t>
+  </si>
+  <si>
+    <t>CHANGE REQUIRED</t>
+  </si>
+  <si>
+    <t>Change from custom IP ADC_CSn</t>
+  </si>
+  <si>
+    <t>Change from custom IP ADC_MISO_A</t>
+  </si>
+  <si>
+    <t>Change from custom IP ADC_MISO_B</t>
+  </si>
+  <si>
+    <t>Change from custom IP ADC_SCLK</t>
+  </si>
+  <si>
+    <t>Change from AUDIO_EN</t>
+  </si>
+  <si>
+    <t>No change</t>
+  </si>
+  <si>
+    <t>Change from TP7</t>
+  </si>
+  <si>
+    <t>Change from TP6</t>
+  </si>
+  <si>
+    <t>Wired in schematic as DAT1 for uSD but not used - TP15</t>
+  </si>
+  <si>
+    <t>Wired in schematic as DAT1 for uSD but not used - TP16</t>
+  </si>
+  <si>
+    <t>Possible use if necessary may have to completely disconnect form uSD</t>
+  </si>
+  <si>
+    <t>Change from AUDIO_PWM</t>
+  </si>
+  <si>
+    <t>Change name to IOX_GP_SCLK function remains the same</t>
+  </si>
+  <si>
+    <t>Change name to IOX_GP_MOSI function remains the same</t>
+  </si>
+  <si>
+    <t>Change name to IOX_GP_MISO function remains the same</t>
+  </si>
+  <si>
+    <t>Previously not used</t>
+  </si>
+  <si>
+    <t>Change name to IOX_CSn[2]</t>
+  </si>
+  <si>
+    <t>Change name to IOX_CSn[1]</t>
+  </si>
+  <si>
+    <t>Functionally equivlent to IOX_GP_MOSI</t>
+  </si>
+  <si>
+    <t>Functionally equivlent to IOX_GP_SCLK</t>
+  </si>
+  <si>
+    <t>Was previously TP4</t>
   </si>
 </sst>
 </file>
@@ -914,7 +974,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -927,6 +987,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1267,6 +1328,7 @@
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="5" width="15.7109375" customWidth="1"/>
     <col min="6" max="6" width="50.7109375" customWidth="1"/>
+    <col min="7" max="7" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
@@ -1290,10 +1352,10 @@
         <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>132</v>
@@ -1311,6 +1373,9 @@
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
+      <c r="G5" s="10" t="s">
+        <v>259</v>
+      </c>
       <c r="I5" s="3" t="s">
         <v>155</v>
       </c>
@@ -1334,6 +1399,9 @@
       <c r="F6" t="s">
         <v>232</v>
       </c>
+      <c r="G6" t="s">
+        <v>260</v>
+      </c>
       <c r="I6" s="2" t="s">
         <v>156</v>
       </c>
@@ -1357,6 +1425,9 @@
       <c r="F7" t="s">
         <v>159</v>
       </c>
+      <c r="G7" t="s">
+        <v>261</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>157</v>
       </c>
@@ -1380,6 +1451,9 @@
       <c r="F8" t="s">
         <v>233</v>
       </c>
+      <c r="G8" t="s">
+        <v>262</v>
+      </c>
       <c r="I8" t="s">
         <v>163</v>
       </c>
@@ -1406,6 +1480,9 @@
       <c r="F9" t="s">
         <v>234</v>
       </c>
+      <c r="G9" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1418,7 +1495,7 @@
         <v>105</v>
       </c>
       <c r="I10" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1432,7 +1509,7 @@
         <v>106</v>
       </c>
       <c r="I11" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1454,6 +1531,9 @@
       <c r="F12" t="s">
         <v>235</v>
       </c>
+      <c r="G12" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1466,13 +1546,16 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F13" t="s">
         <v>172</v>
+      </c>
+      <c r="G13" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1494,6 +1577,9 @@
       <c r="F14" t="s">
         <v>236</v>
       </c>
+      <c r="G14" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1514,6 +1600,9 @@
       <c r="F15" t="s">
         <v>161</v>
       </c>
+      <c r="G15" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1526,7 +1615,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>102</v>
       </c>
@@ -1537,7 +1626,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>168</v>
       </c>
@@ -1547,7 +1636,7 @@
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1558,7 +1647,7 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>145</v>
@@ -1567,7 +1656,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1578,7 +1667,7 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>146</v>
@@ -1587,7 +1676,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1598,7 +1687,7 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>149</v>
@@ -1607,7 +1696,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1618,7 +1707,7 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>151</v>
@@ -1627,7 +1716,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>109</v>
       </c>
@@ -1638,7 +1727,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -1649,7 +1738,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1660,13 +1749,16 @@
         <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F25" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="G25" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1677,13 +1769,16 @@
         <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F26" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+      <c r="G26" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1694,7 +1789,7 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>153</v>
@@ -1703,7 +1798,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1722,8 +1817,11 @@
       <c r="F28" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>111</v>
       </c>
@@ -1734,7 +1832,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>112</v>
       </c>
@@ -1745,7 +1843,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>166</v>
       </c>
@@ -1755,7 +1853,7 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1766,7 +1864,7 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>219</v>
@@ -1774,8 +1872,11 @@
       <c r="F32" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -1786,7 +1887,7 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>220</v>
@@ -1794,8 +1895,11 @@
       <c r="F33" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1806,16 +1910,19 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F34" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -1826,16 +1933,16 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F35" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>117</v>
       </c>
@@ -1846,7 +1953,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>118</v>
       </c>
@@ -1857,7 +1964,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1871,13 +1978,16 @@
         <v>224</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F38" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -1895,7 +2005,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -1912,8 +2022,11 @@
       <c r="F40" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1930,8 +2043,11 @@
       <c r="F41" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>119</v>
       </c>
@@ -1942,7 +2058,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>120</v>
       </c>
@@ -1953,7 +2069,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>167</v>
       </c>
@@ -1963,7 +2079,7 @@
       <c r="E44" s="8"/>
       <c r="F44" s="8"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -1983,7 +2099,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -2003,7 +2119,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -2023,7 +2139,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -2042,8 +2158,11 @@
       <c r="F48" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>125</v>
       </c>
@@ -2054,7 +2173,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -2065,7 +2184,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -2076,7 +2195,7 @@
         <v>71</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>143</v>
@@ -2085,7 +2204,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -2096,7 +2215,7 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>144</v>
@@ -2105,7 +2224,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -2116,16 +2235,19 @@
         <v>73</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>169</v>
       </c>
       <c r="F53" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+        <v>252</v>
+      </c>
+      <c r="G53" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -2144,8 +2266,11 @@
       <c r="F54" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>127</v>
       </c>
@@ -2156,7 +2281,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>128</v>
       </c>
@@ -2167,7 +2292,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>170</v>
       </c>
@@ -2177,7 +2302,7 @@
       <c r="E57" s="8"/>
       <c r="F57" s="8"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>66</v>
       </c>
@@ -2195,7 +2320,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
@@ -2213,7 +2338,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -2231,7 +2356,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>71</v>
       </c>
@@ -2249,7 +2374,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>73</v>
       </c>
@@ -2267,7 +2392,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>130</v>
       </c>
@@ -2285,7 +2410,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>181</v>
       </c>

</xml_diff>

<commit_message>
Update to PCB - no real change - release for fab
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -10,12 +10,13 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D09CBD-13FA-4135-8F34-5E553F38B417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -983,11 +984,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1365,15 +1366,15 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="10" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="9" t="s">
         <v>259</v>
       </c>
       <c r="I5" s="3" t="s">
@@ -1627,14 +1628,14 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1844,14 +1845,14 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -2070,14 +2071,14 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -2194,7 +2195,7 @@
       <c r="C51" t="s">
         <v>71</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="8" t="s">
         <v>249</v>
       </c>
       <c r="E51" s="3" t="s">
@@ -2293,14 +2294,14 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
+      <c r="A57" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B57" s="8"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="8"/>
-      <c r="E57" s="8"/>
-      <c r="F57" s="8"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">

</xml_diff>

<commit_message>
Changes to PL Block Diagram and constraints file as well as changes to FW to account for change in HW and make work so I can beging working on FW. Currently debugging encoder rotation - overall boot process is flaky - sometimes having failures with IO expander
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA_P2\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D09CBD-13FA-4135-8F34-5E553F38B417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB70847-3B1B-41D3-B9B5-36FF5C6CD047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="305">
   <si>
     <t>G13</t>
   </si>
@@ -561,21 +560,12 @@
     <t>IO Expander common Reset (active low)</t>
   </si>
   <si>
-    <t>UI_CSn[1]</t>
-  </si>
-  <si>
     <t>IO Expander 1 chip select (active low)</t>
   </si>
   <si>
-    <t>UI_CSn[2]</t>
-  </si>
-  <si>
     <t>IO Expander 2 chip select (active low)</t>
   </si>
   <si>
-    <t>IO Expander common SPI MISO</t>
-  </si>
-  <si>
     <t>IOX_2_IRQ</t>
   </si>
   <si>
@@ -618,9 +608,6 @@
     <t>TEST_IRQ (Timer 1 IRQ input to interrupt controller)</t>
   </si>
   <si>
-    <t>ADC_IP_IRQ</t>
-  </si>
-  <si>
     <t>CK_IO6</t>
   </si>
   <si>
@@ -633,12 +620,6 @@
     <t>T16</t>
   </si>
   <si>
-    <t>ADC_IP_IRQ: Primary IRQ for ADC IP 7476Ax2</t>
-  </si>
-  <si>
-    <t>ADC_IRQ_N_DONE: N number of conversions done - indirect IRQ for ADC IP 7476Ax2</t>
-  </si>
-  <si>
     <t>U16</t>
   </si>
   <si>
@@ -651,9 +632,6 @@
     <t>CK_IO0</t>
   </si>
   <si>
-    <t>TEST_IO_1</t>
-  </si>
-  <si>
     <t>MB_CLK</t>
   </si>
   <si>
@@ -675,9 +653,6 @@
     <t>UI_CSn - not used for display - display uses JD1 - J4.1 for CSn</t>
   </si>
   <si>
-    <t>UI_CSn</t>
-  </si>
-  <si>
     <t>ADC_IRQ_N_DONE</t>
   </si>
   <si>
@@ -690,18 +665,6 @@
     <t>DIGILENT ARTY A7 TO IMR-107-SCH PIN MAP</t>
   </si>
   <si>
-    <t>IO Expander &amp; GP common SPI SCLK</t>
-  </si>
-  <si>
-    <t>IO Expander &amp; GP common SPI MOSI</t>
-  </si>
-  <si>
-    <t>IOX_GP_SCLK</t>
-  </si>
-  <si>
-    <t>IOX_GP_MOSI</t>
-  </si>
-  <si>
     <t>Programmable Waveform Generator Chip Select / FSYNC</t>
   </si>
   <si>
@@ -804,9 +767,6 @@
     <t>gpio2_io_o_0[8]</t>
   </si>
   <si>
-    <t>IOX_GP_MISO</t>
-  </si>
-  <si>
     <t>X_SCLK</t>
   </si>
   <si>
@@ -880,6 +840,117 @@
   </si>
   <si>
     <t>Was previously TP4</t>
+  </si>
+  <si>
+    <t>J4.14</t>
+  </si>
+  <si>
+    <t>J4.16</t>
+  </si>
+  <si>
+    <t>CK_IO26</t>
+  </si>
+  <si>
+    <t>CK_IO27</t>
+  </si>
+  <si>
+    <t>CK_IO28</t>
+  </si>
+  <si>
+    <t>CK_IO29</t>
+  </si>
+  <si>
+    <t>CK_IO30</t>
+  </si>
+  <si>
+    <t>CK_IO31</t>
+  </si>
+  <si>
+    <t>CK_IO32</t>
+  </si>
+  <si>
+    <t>CK_IO33</t>
+  </si>
+  <si>
+    <t>U11</t>
+  </si>
+  <si>
+    <t>V16</t>
+  </si>
+  <si>
+    <t>M13</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>R11</t>
+  </si>
+  <si>
+    <t>R13</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>P15</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[0]</t>
+  </si>
+  <si>
+    <t>TIMER_1_OUTPUT</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[1]</t>
+  </si>
+  <si>
+    <t>TIMER_2_OUTPUT</t>
+  </si>
+  <si>
+    <t>IOX_CSn[0]</t>
+  </si>
+  <si>
+    <t>IOX_SCLK</t>
+  </si>
+  <si>
+    <t>IOX_MOSI</t>
+  </si>
+  <si>
+    <t>X_MISO</t>
+  </si>
+  <si>
+    <t>Common SPI SCLK for IO Expanders (x2), Display, and Waveform Generator</t>
+  </si>
+  <si>
+    <t>Common SPI MOSI for IO Expanders (x2), Display, and Waveform Generator</t>
+  </si>
+  <si>
+    <t>Common SPI MISO for IO Expanders (x2), NOT USED BY: Display, and Waveform Generator</t>
+  </si>
+  <si>
+    <t>IOX_RESET</t>
+  </si>
+  <si>
+    <t>IOX_CSn[1]</t>
+  </si>
+  <si>
+    <t>IOX_CSn[2]</t>
+  </si>
+  <si>
+    <t>IOX_CSn[3]</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[9]</t>
+  </si>
+  <si>
+    <t>Temp placement for gpio2_io_o_0[5] to get compile</t>
+  </si>
+  <si>
+    <t>TEST_IO_0 - Used in ADC ISR as toggle</t>
+  </si>
+  <si>
+    <t>TEST_IO_1 - Presently not used</t>
   </si>
 </sst>
 </file>
@@ -975,7 +1046,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -989,6 +1060,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1323,23 +1396,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AF3F25-4127-44F5-ACE1-35E82582D3CE}">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="50.7109375" customWidth="1"/>
+    <col min="6" max="6" width="60.7109375" customWidth="1"/>
     <col min="7" max="7" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -1353,10 +1426,10 @@
         <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>132</v>
@@ -1375,7 +1448,7 @@
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="9" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>155</v>
@@ -1392,16 +1465,16 @@
         <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="F6" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="G6" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>156</v>
@@ -1427,7 +1500,7 @@
         <v>159</v>
       </c>
       <c r="G7" t="s">
-        <v>261</v>
+        <v>248</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>157</v>
@@ -1444,16 +1517,16 @@
         <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="F8" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="G8" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="I8" t="s">
         <v>163</v>
@@ -1473,16 +1546,16 @@
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="F9" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="G9" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1496,7 +1569,7 @@
         <v>105</v>
       </c>
       <c r="I10" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1510,7 +1583,7 @@
         <v>106</v>
       </c>
       <c r="I11" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1524,16 +1597,16 @@
         <v>95</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="F12" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="G12" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1547,16 +1620,16 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="F13" t="s">
         <v>172</v>
       </c>
       <c r="G13" t="s">
-        <v>265</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1570,16 +1643,16 @@
         <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="F14" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="G14" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1602,7 +1675,7 @@
         <v>161</v>
       </c>
       <c r="G15" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1648,7 +1721,7 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>145</v>
@@ -1668,7 +1741,7 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>146</v>
@@ -1688,7 +1761,7 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>149</v>
@@ -1708,7 +1781,7 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>151</v>
@@ -1750,13 +1823,13 @@
         <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="F25" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="G25" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1770,13 +1843,13 @@
         <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="F26" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
       <c r="G26" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1790,13 +1863,13 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>153</v>
       </c>
       <c r="F27" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1810,16 +1883,16 @@
         <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>222</v>
+        <v>300</v>
       </c>
       <c r="F28" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="G28" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1865,16 +1938,16 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>219</v>
+        <v>291</v>
       </c>
       <c r="F32" t="s">
-        <v>217</v>
+        <v>294</v>
       </c>
       <c r="G32" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1888,16 +1961,16 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>220</v>
+        <v>292</v>
       </c>
       <c r="F33" t="s">
-        <v>218</v>
+        <v>295</v>
       </c>
       <c r="G33" t="s">
-        <v>273</v>
+        <v>260</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1911,16 +1984,16 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>255</v>
+        <v>293</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>255</v>
+        <v>293</v>
       </c>
       <c r="F34" t="s">
-        <v>178</v>
+        <v>296</v>
       </c>
       <c r="G34" t="s">
-        <v>274</v>
+        <v>261</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1934,13 +2007,16 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="F35" t="s">
         <v>173</v>
+      </c>
+      <c r="G35" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1976,16 +2052,16 @@
         <v>79</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="F38" t="s">
         <v>171</v>
       </c>
       <c r="G38" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1999,11 +2075,11 @@
         <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -2016,15 +2092,14 @@
       <c r="C40" t="s">
         <v>81</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E40" s="2"/>
+      <c r="E40" s="2" t="s">
+        <v>299</v>
+      </c>
       <c r="F40" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G40" t="s">
-        <v>276</v>
+        <v>263</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -2037,15 +2112,14 @@
       <c r="C41" t="s">
         <v>82</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F41" t="s">
         <v>174</v>
       </c>
-      <c r="E41" s="2"/>
-      <c r="F41" t="s">
-        <v>175</v>
-      </c>
       <c r="G41" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -2160,7 +2234,7 @@
         <v>140</v>
       </c>
       <c r="G48" t="s">
-        <v>278</v>
+        <v>265</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -2196,13 +2270,13 @@
         <v>71</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F51" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -2216,13 +2290,13 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -2236,16 +2310,16 @@
         <v>73</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>169</v>
       </c>
       <c r="F53" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="G53" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -2268,7 +2342,7 @@
         <v>142</v>
       </c>
       <c r="G54" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -2308,35 +2382,29 @@
         <v>66</v>
       </c>
       <c r="B58" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C58" t="s">
-        <v>203</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="E58" s="2"/>
-      <c r="F58" t="s">
-        <v>204</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C59" t="s">
+        <v>195</v>
+      </c>
+      <c r="E59" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="F59" t="s">
         <v>201</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E59" s="2"/>
-      <c r="F59" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -2344,17 +2412,16 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C60" t="s">
-        <v>183</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="E60" s="5"/>
+        <v>180</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>200</v>
+      </c>
       <c r="F60" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -2362,17 +2429,16 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C61" t="s">
-        <v>186</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="E61" s="5"/>
+        <v>183</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>188</v>
+      </c>
       <c r="F61" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
@@ -2380,17 +2446,16 @@
         <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C62" t="s">
-        <v>187</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E62" s="2"/>
+        <v>184</v>
+      </c>
+      <c r="E62" s="11" t="s">
+        <v>205</v>
+      </c>
       <c r="F62" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -2398,53 +2463,162 @@
         <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C63" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E63" s="2"/>
+        <v>290</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>290</v>
+      </c>
       <c r="F63" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B64" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C64" t="s">
-        <v>194</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="E64" s="2"/>
-      <c r="F64" t="s">
-        <v>198</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="D64" s="11"/>
+      <c r="E64" s="11"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B65" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C65" t="s">
-        <v>195</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="E65" s="2"/>
-      <c r="F65" t="s">
+        <v>191</v>
+      </c>
+      <c r="E65" s="11"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>67</v>
+      </c>
+      <c r="B66" t="s">
+        <v>278</v>
+      </c>
+      <c r="C66" t="s">
+        <v>270</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="F66" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" t="s">
+        <v>279</v>
+      </c>
+      <c r="C67" t="s">
+        <v>271</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="F67" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>129</v>
+      </c>
+      <c r="B68" t="s">
+        <v>280</v>
+      </c>
+      <c r="C68" t="s">
+        <v>272</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="F68" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69" t="s">
+        <v>281</v>
+      </c>
+      <c r="C69" t="s">
+        <v>273</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>199</v>
+      </c>
+      <c r="F69" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70" t="s">
+        <v>282</v>
+      </c>
+      <c r="C70" t="s">
+        <v>274</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F70" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>131</v>
+      </c>
+      <c r="B71" t="s">
+        <v>283</v>
+      </c>
+      <c r="C71" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>268</v>
+      </c>
+      <c r="B72" t="s">
+        <v>284</v>
+      </c>
+      <c r="C72" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>269</v>
+      </c>
+      <c r="B73" t="s">
+        <v>285</v>
+      </c>
+      <c r="C73" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Many changes to refactor the way the generic spi tx rx function works - a few more changes to go
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA_P2\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB70847-3B1B-41D3-B9B5-36FF5C6CD047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9F3CF7-3791-4B4A-952E-B4786659F287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="300">
   <si>
     <t>G13</t>
   </si>
@@ -605,9 +605,6 @@
     <t>MB_RESET</t>
   </si>
   <si>
-    <t>TEST_IRQ (Timer 1 IRQ input to interrupt controller)</t>
-  </si>
-  <si>
     <t>CK_IO6</t>
   </si>
   <si>
@@ -635,15 +632,9 @@
     <t>MB_CLK</t>
   </si>
   <si>
-    <t>gpio2_io_o_0[10]</t>
-  </si>
-  <si>
     <t>TEST_IRQ</t>
   </si>
   <si>
-    <t>MicroBlaze Clock</t>
-  </si>
-  <si>
     <t>MicroBlaze Reset</t>
   </si>
   <si>
@@ -665,9 +656,6 @@
     <t>DIGILENT ARTY A7 TO IMR-107-SCH PIN MAP</t>
   </si>
   <si>
-    <t>Programmable Waveform Generator Chip Select / FSYNC</t>
-  </si>
-  <si>
     <t>FSYNC</t>
   </si>
   <si>
@@ -776,72 +764,18 @@
     <t>gpio2_io_o_0[7]</t>
   </si>
   <si>
-    <t>CHANGE REQUIRED</t>
-  </si>
-  <si>
-    <t>Change from custom IP ADC_CSn</t>
-  </si>
-  <si>
-    <t>Change from custom IP ADC_MISO_A</t>
-  </si>
-  <si>
-    <t>Change from custom IP ADC_MISO_B</t>
-  </si>
-  <si>
-    <t>Change from custom IP ADC_SCLK</t>
-  </si>
-  <si>
-    <t>Change from AUDIO_EN</t>
-  </si>
-  <si>
-    <t>No change</t>
-  </si>
-  <si>
-    <t>Change from TP7</t>
-  </si>
-  <si>
-    <t>Change from TP6</t>
-  </si>
-  <si>
     <t>Wired in schematic as DAT1 for uSD but not used - TP15</t>
   </si>
   <si>
     <t>Wired in schematic as DAT1 for uSD but not used - TP16</t>
   </si>
   <si>
-    <t>Possible use if necessary may have to completely disconnect form uSD</t>
-  </si>
-  <si>
-    <t>Change from AUDIO_PWM</t>
-  </si>
-  <si>
-    <t>Change name to IOX_GP_SCLK function remains the same</t>
-  </si>
-  <si>
-    <t>Change name to IOX_GP_MOSI function remains the same</t>
-  </si>
-  <si>
-    <t>Change name to IOX_GP_MISO function remains the same</t>
-  </si>
-  <si>
-    <t>Previously not used</t>
-  </si>
-  <si>
-    <t>Change name to IOX_CSn[2]</t>
-  </si>
-  <si>
-    <t>Change name to IOX_CSn[1]</t>
-  </si>
-  <si>
     <t>Functionally equivlent to IOX_GP_MOSI</t>
   </si>
   <si>
     <t>Functionally equivlent to IOX_GP_SCLK</t>
   </si>
   <si>
-    <t>Was previously TP4</t>
-  </si>
-  <si>
     <t>J4.14</t>
   </si>
   <si>
@@ -950,7 +884,58 @@
     <t>TEST_IO_0 - Used in ADC ISR as toggle</t>
   </si>
   <si>
-    <t>TEST_IO_1 - Presently not used</t>
+    <t>WAVEFORM_GEN_CS</t>
+  </si>
+  <si>
+    <t>Could not get the chip select 3 of AXI QSPIO 0 to so I used gpio2_io_o_0[10]</t>
+  </si>
+  <si>
+    <t>Waveform Generator Chip Select / FSYNC</t>
+  </si>
+  <si>
+    <t>FIRMWARE</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>SIG_SEL</t>
+  </si>
+  <si>
+    <t>AUDIO_EN</t>
+  </si>
+  <si>
+    <t>DISPLAY_CS</t>
+  </si>
+  <si>
+    <t>DISPLAY_CMD_DATA</t>
+  </si>
+  <si>
+    <t>DISPLAY_RESET_RUN</t>
+  </si>
+  <si>
+    <t>TIIMER_1_OUTPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST_IO_0 </t>
+  </si>
+  <si>
+    <t>Could not get</t>
+  </si>
+  <si>
+    <t>Temp placement for</t>
+  </si>
+  <si>
+    <t>For test only MicroBlaze Clock</t>
+  </si>
+  <si>
+    <t>For test only TEST_IRQ (Timer 1 IRQ input to interrupt controller)</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>Can possibly be used if so may have to completely disconnect form uSD</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1031,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1057,11 +1042,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1396,26 +1386,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AF3F25-4127-44F5-ACE1-35E82582D3CE}">
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
-    <col min="7" max="7" width="40.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="60.7109375" customWidth="1"/>
+    <col min="8" max="8" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D3" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>154</v>
       </c>
@@ -1426,35 +1424,40 @@
         <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="I4" t="s">
+      <c r="H4" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="J4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="9"/>
+      <c r="J5" s="3" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1465,22 +1468,20 @@
         <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" t="s">
         <v>216</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="F6" t="s">
-        <v>220</v>
-      </c>
-      <c r="G6" t="s">
-        <v>247</v>
-      </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1496,17 +1497,15 @@
       <c r="E7" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="3"/>
+      <c r="G7" t="s">
         <v>159</v>
       </c>
-      <c r="G7" t="s">
-        <v>248</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1517,25 +1516,23 @@
         <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" t="s">
         <v>217</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F8" t="s">
-        <v>221</v>
-      </c>
-      <c r="G8" t="s">
-        <v>249</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>163</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1546,19 +1543,17 @@
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" t="s">
         <v>218</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="F9" t="s">
-        <v>222</v>
-      </c>
-      <c r="G9" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>99</v>
       </c>
@@ -1568,11 +1563,11 @@
       <c r="D10" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I10" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J10" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>100</v>
       </c>
@@ -1582,11 +1577,11 @@
       <c r="D11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="I11" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J11" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1597,19 +1592,17 @@
         <v>95</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="F12" t="s">
-        <v>223</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="F12" s="5"/>
       <c r="G12" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1620,19 +1613,19 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="F13" t="s">
+        <v>241</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="G13" t="s">
         <v>172</v>
       </c>
-      <c r="G13" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1643,19 +1636,17 @@
         <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F14" t="s">
-        <v>224</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="F14" s="2"/>
       <c r="G14" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1671,14 +1662,12 @@
       <c r="E15" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2"/>
+      <c r="G15" t="s">
         <v>161</v>
       </c>
-      <c r="G15" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -1689,7 +1678,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>102</v>
       </c>
@@ -1700,17 +1689,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1721,16 +1711,17 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="2"/>
+      <c r="G19" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1741,16 +1732,17 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2"/>
+      <c r="G20" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1761,16 +1753,17 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="3"/>
+      <c r="G21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1781,16 +1774,17 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="2"/>
+      <c r="G22" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>109</v>
       </c>
@@ -1801,7 +1795,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -1812,7 +1806,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1823,16 +1817,16 @@
         <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>232</v>
-      </c>
-      <c r="F25" t="s">
-        <v>255</v>
+        <v>228</v>
       </c>
       <c r="G25" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+      <c r="H25" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1843,16 +1837,16 @@
         <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>233</v>
-      </c>
-      <c r="F26" t="s">
-        <v>256</v>
+        <v>229</v>
       </c>
       <c r="G26" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+      <c r="H26" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1863,16 +1857,17 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F27" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F27" s="3"/>
+      <c r="G27" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1883,19 +1878,19 @@
         <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="F28" t="s">
-        <v>209</v>
+        <v>266</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>282</v>
       </c>
       <c r="G28" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>111</v>
       </c>
@@ -1906,7 +1901,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>112</v>
       </c>
@@ -1917,17 +1912,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1938,19 +1934,17 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="F32" t="s">
-        <v>294</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="F32" s="2"/>
       <c r="G32" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -1961,19 +1955,17 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="F33" t="s">
-        <v>295</v>
-      </c>
+        <v>270</v>
+      </c>
+      <c r="F33" s="2"/>
       <c r="G33" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1984,19 +1976,17 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="F34" t="s">
-        <v>296</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="F34" s="3"/>
       <c r="G34" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -2007,19 +1997,19 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F35" t="s">
+        <v>238</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G35" t="s">
         <v>173</v>
       </c>
-      <c r="G35" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>117</v>
       </c>
@@ -2030,7 +2020,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>118</v>
       </c>
@@ -2041,7 +2031,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -2052,19 +2042,19 @@
         <v>79</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="F38" t="s">
+        <v>237</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G38" t="s">
         <v>171</v>
       </c>
-      <c r="G38" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -2078,11 +2068,12 @@
         <v>176</v>
       </c>
       <c r="E39" s="3"/>
-      <c r="F39" t="s">
+      <c r="F39" s="3"/>
+      <c r="G39" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -2093,16 +2084,14 @@
         <v>81</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="F40" t="s">
+        <v>277</v>
+      </c>
+      <c r="F40" s="2"/>
+      <c r="G40" t="s">
         <v>175</v>
       </c>
-      <c r="G40" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -2113,16 +2102,14 @@
         <v>82</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="F41" t="s">
+        <v>276</v>
+      </c>
+      <c r="F41" s="2"/>
+      <c r="G41" t="s">
         <v>174</v>
       </c>
-      <c r="G41" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>119</v>
       </c>
@@ -2133,7 +2120,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>120</v>
       </c>
@@ -2144,17 +2131,18 @@
         <v>106</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -2170,11 +2158,14 @@
       <c r="E45" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="G45" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -2190,11 +2181,14 @@
       <c r="E46" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G46" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -2210,11 +2204,14 @@
       <c r="E47" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="G47" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -2230,14 +2227,15 @@
       <c r="E48" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="2"/>
+      <c r="G48" t="s">
         <v>140</v>
       </c>
-      <c r="G48" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>125</v>
       </c>
@@ -2248,7 +2246,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -2259,7 +2257,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -2270,16 +2268,17 @@
         <v>71</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="F51" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F51" s="3"/>
+      <c r="G51" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -2290,16 +2289,17 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="F52" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F52" s="2"/>
+      <c r="G52" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -2310,19 +2310,17 @@
         <v>73</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F53" t="s">
-        <v>240</v>
-      </c>
+      <c r="F53" s="2"/>
       <c r="G53" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -2338,14 +2336,15 @@
       <c r="E54" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="2"/>
+      <c r="G54" t="s">
         <v>142</v>
       </c>
-      <c r="G54" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H54" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>127</v>
       </c>
@@ -2356,7 +2355,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>128</v>
       </c>
@@ -2367,47 +2366,46 @@
         <v>106</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>66</v>
       </c>
       <c r="B58" t="s">
+        <v>195</v>
+      </c>
+      <c r="C58" t="s">
         <v>196</v>
       </c>
-      <c r="C58" t="s">
-        <v>197</v>
-      </c>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
       <c r="B59" t="s">
+        <v>193</v>
+      </c>
+      <c r="C59" t="s">
         <v>194</v>
       </c>
-      <c r="C59" t="s">
-        <v>195</v>
-      </c>
-      <c r="E59" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="F59" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E59" t="s">
+        <v>197</v>
+      </c>
+      <c r="G59" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -2417,14 +2415,15 @@
       <c r="C60" t="s">
         <v>180</v>
       </c>
-      <c r="E60" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="F60" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E60" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="F60" s="10"/>
+      <c r="G60" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>71</v>
       </c>
@@ -2434,14 +2433,15 @@
       <c r="C61" t="s">
         <v>183</v>
       </c>
-      <c r="E61" s="12" t="s">
+      <c r="E61" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="F61" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F61" s="10"/>
+      <c r="G61" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>73</v>
       </c>
@@ -2451,14 +2451,14 @@
       <c r="C62" t="s">
         <v>184</v>
       </c>
-      <c r="E62" s="11" t="s">
-        <v>205</v>
-      </c>
-      <c r="F62" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E62" t="s">
+        <v>202</v>
+      </c>
+      <c r="G62" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>130</v>
       </c>
@@ -2469,166 +2469,181 @@
         <v>187</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="F63" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="F63" s="2"/>
+      <c r="G63" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>178</v>
       </c>
       <c r="B64" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C64" t="s">
-        <v>190</v>
-      </c>
-      <c r="D64" s="11"/>
-      <c r="E64" s="11"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>179</v>
       </c>
       <c r="B65" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C65" t="s">
-        <v>191</v>
-      </c>
-      <c r="E65" s="11"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="C66" t="s">
-        <v>270</v>
+        <v>248</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F66" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G66" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C67" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="F67" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+        <v>266</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="G67" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>129</v>
       </c>
       <c r="B68" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="C68" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="F68" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+        <v>279</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="G68" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>72</v>
       </c>
       <c r="B69" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C69" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F69" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+        <v>278</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G69" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C70" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F70" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G70" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>131</v>
       </c>
       <c r="B71" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="C71" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="B72" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="C72" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="B73" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C73" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="A57:F57"/>
+  <mergeCells count="6">
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A57:G57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>